<commit_message>
restructured the code a little bit
</commit_message>
<xml_diff>
--- a/Trip_SFO_to_ZRH_2026-09-05.xlsx
+++ b/Trip_SFO_to_ZRH_2026-09-05.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Flights" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hotels" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -527,7 +528,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>This is the best option by far. It's a direct flight, has the shortest travel time (11 hours), and arrives at a reasonable early evening hour (18:10), which is crucial for settling in with a 3-year-old. The higher price is justified by the significant convenience.</t>
+          <t>This is the clear winner for parents with a toddler. It's a direct flight, has the shortest travel time (11 hours), and arrives at a very reasonable 18:10 (6:10 PM), allowing plenty of time to get to the accommodation and settle in before bedtime. The higher price is well worth the convenience.</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -590,11 +591,11 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>While cheaper, this flight has one layover and a longer total travel time (14.2 hours) compared to Swiss Air. The arrival time of 21:45 is late for a toddler, making it more challenging to get settled for the night, but it's still better than the British Airways option.</t>
+          <t>While it has a layover and a longer duration (14.2 hours) compared to Swiss Air, it's still a decent option. The arrival time of 21:45 (9:45 PM) is late but manageable. The lower price makes it somewhat attractive, but convenience is prioritized.</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -657,11 +658,11 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Despite being the cheapest, this is the least convenient option for a family with a toddler. It has one layover, the longest travel duration (15.5 hours), and a very late arrival time of 23:50, which would be extremely difficult for a 3-year-old and their parents.</t>
+          <t>This flight is the least convenient. It has a layover, the longest travel time (15.5 hours), and a very late arrival time of 23:50 (11:50 PM). Arriving almost at midnight after a long travel day with a toddler will be extremely challenging, making the lowest price insufficient to compensate for the inconvenience.</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -692,6 +693,118 @@
         <is>
           <t>23:50</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>hotel_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>price_per_night</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>rating</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>distance_to_center_km</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>crib_available</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>kitchen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Central Family Suites</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>260</v>
+      </c>
+      <c r="C2" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Budget City Stay</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>155</v>
+      </c>
+      <c r="C3" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Parkside Aparthotel</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>220</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>